<commit_message>
Bake computed values into projections workbook
Viewers that do not recalculate formulas (Drive preview, mobile) showed
zeros; projected figures are now stored as static values.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PixbgqB4jdMpq9cU3Yt7Dw
</commit_message>
<xml_diff>
--- a/projections/PROJECTIONS_FY2026-27_BS_PL_set2.xlsx
+++ b/projections/PROJECTIONS_FY2026-27_BS_PL_set2.xlsx
@@ -567,6 +567,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -833,10 +834,11 @@
       </c>
       <c r="C22" s="5" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Note: Change the growth rate in cell C6 — the projected P&amp;L and Balance Sheet recalculate automatically.</t>
+          <t>Note: Figures are computed at 10% sales growth and stored as values so they display in any viewer.</t>
         </is>
       </c>
     </row>
@@ -930,13 +932,11 @@
       <c r="C6" s="11" t="n">
         <v>4898238075.54</v>
       </c>
-      <c r="D6" s="11">
-        <f>C6*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E6" s="12">
-        <f>IFERROR(D6/C6-1,"")</f>
-        <v/>
+      <c r="D6" s="11" t="n">
+        <v>5388061883.094001</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
@@ -958,13 +958,11 @@
       <c r="C7" s="11" t="n">
         <v>9993615.65</v>
       </c>
-      <c r="D7" s="11">
-        <f>C7</f>
-        <v/>
-      </c>
-      <c r="E7" s="12">
-        <f>IFERROR(D7/C7-1,"")</f>
-        <v/>
+      <c r="D7" s="11" t="n">
+        <v>9993615.65</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
@@ -983,17 +981,14 @@
           <t>Total Income (I+II)</t>
         </is>
       </c>
-      <c r="C8" s="16">
-        <f>SUM(C6:C7)</f>
-        <v/>
-      </c>
-      <c r="D8" s="16">
-        <f>SUM(D6:D7)</f>
-        <v/>
-      </c>
-      <c r="E8" s="17">
-        <f>IFERROR(D8/C8-1,"")</f>
-        <v/>
+      <c r="C8" s="16" t="n">
+        <v>4908231691.19</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>5398055498.744</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>0.09979639071097779</v>
       </c>
       <c r="F8" s="18" t="inlineStr"/>
     </row>
@@ -1023,13 +1018,11 @@
       <c r="C10" s="11" t="n">
         <v>129055957.47</v>
       </c>
-      <c r="D10" s="11">
-        <f>C10*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E10" s="12">
-        <f>IFERROR(D10/C10-1,"")</f>
-        <v/>
+      <c r="D10" s="11" t="n">
+        <v>141961553.217</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
@@ -1067,13 +1060,11 @@
       <c r="C12" s="11" t="n">
         <v>4143800770.32</v>
       </c>
-      <c r="D12" s="11">
-        <f>C12*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E12" s="12">
-        <f>IFERROR(D12/C12-1,"")</f>
-        <v/>
+      <c r="D12" s="11" t="n">
+        <v>4558180847.352</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
@@ -1091,13 +1082,11 @@
       <c r="C13" s="11" t="n">
         <v>34403667</v>
       </c>
-      <c r="D13" s="11">
-        <f>C13*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E13" s="12">
-        <f>IFERROR(D13/C13-1,"")</f>
-        <v/>
+      <c r="D13" s="11" t="n">
+        <v>37844033.7</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
@@ -1115,13 +1104,11 @@
       <c r="C14" s="11" t="n">
         <v>26150367</v>
       </c>
-      <c r="D14" s="11">
-        <f>C14*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E14" s="12">
-        <f>IFERROR(D14/C14-1,"")</f>
-        <v/>
+      <c r="D14" s="11" t="n">
+        <v>28765403.7</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -1139,13 +1126,11 @@
       <c r="C15" s="11" t="n">
         <v>433672461.96</v>
       </c>
-      <c r="D15" s="11">
-        <f>C15*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E15" s="12">
-        <f>IFERROR(D15/C15-1,"")</f>
-        <v/>
+      <c r="D15" s="11" t="n">
+        <v>477039708.156</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
@@ -1160,17 +1145,14 @@
           <t>Total expenses</t>
         </is>
       </c>
-      <c r="C16" s="16">
-        <f>SUM(C10:C15)</f>
-        <v/>
-      </c>
-      <c r="D16" s="16">
-        <f>SUM(D10:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="17">
-        <f>D16/C16-1</f>
-        <v/>
+      <c r="C16" s="16" t="n">
+        <v>4767109448.75</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <v>5243791546.125</v>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>0.09999394863904221</v>
       </c>
       <c r="F16" s="18" t="inlineStr"/>
     </row>
@@ -1185,17 +1167,14 @@
           <t>Profit Before Tax (III-IV)</t>
         </is>
       </c>
-      <c r="C17" s="21">
-        <f>C8-C16</f>
-        <v/>
-      </c>
-      <c r="D17" s="21">
-        <f>D8-D16</f>
-        <v/>
-      </c>
-      <c r="E17" s="22">
-        <f>D17/C17-1</f>
-        <v/>
+      <c r="C17" s="21" t="n">
+        <v>141122242.4399996</v>
+      </c>
+      <c r="D17" s="21" t="n">
+        <v>154263952.6190004</v>
+      </c>
+      <c r="E17" s="22" t="n">
+        <v>0.09312288376219824</v>
       </c>
       <c r="F17" s="23" t="inlineStr"/>
     </row>
@@ -1213,13 +1192,11 @@
       <c r="C18" s="11" t="n">
         <v>-29662103</v>
       </c>
-      <c r="D18" s="11">
-        <f>ROUND(D17*Assumptions!$C$14,0)</f>
-        <v/>
-      </c>
-      <c r="E18" s="12">
-        <f>IFERROR(D18/C18-1,"")</f>
-        <v/>
+      <c r="D18" s="11" t="n">
+        <v>38825152</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>-2.308914340969014</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
@@ -1241,13 +1218,11 @@
       <c r="C19" s="16" t="n">
         <v>170784345.44</v>
       </c>
-      <c r="D19" s="16">
-        <f>D17-D18</f>
-        <v/>
-      </c>
-      <c r="E19" s="17">
-        <f>D19/C19-1</f>
-        <v/>
+      <c r="D19" s="16" t="n">
+        <v>115438800.6190004</v>
+      </c>
+      <c r="E19" s="17" t="n">
+        <v>-0.3240668497947523</v>
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
@@ -1262,13 +1237,11 @@
           <t>PBT margin</t>
         </is>
       </c>
-      <c r="C21" s="12">
-        <f>C17/C6</f>
-        <v/>
-      </c>
-      <c r="D21" s="12">
-        <f>D17/D6</f>
-        <v/>
+      <c r="C21" s="12" t="n">
+        <v>0.02881081733138129</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>0.02863069429529585</v>
       </c>
       <c r="E21" s="9" t="n"/>
       <c r="F21" s="13" t="inlineStr"/>
@@ -1280,13 +1253,11 @@
           <t>PAT margin</t>
         </is>
       </c>
-      <c r="C22" s="12">
-        <f>C19/C6</f>
-        <v/>
-      </c>
-      <c r="D22" s="12">
-        <f>D19/D6</f>
-        <v/>
+      <c r="C22" s="12" t="n">
+        <v>0.03486648521492539</v>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>0.02142492107991746</v>
       </c>
       <c r="E22" s="9" t="n"/>
       <c r="F22" s="13" t="inlineStr"/>
@@ -1413,13 +1384,11 @@
       <c r="C8" s="11" t="n">
         <v>200000</v>
       </c>
-      <c r="D8" s="11">
-        <f>C8</f>
-        <v/>
-      </c>
-      <c r="E8" s="12">
-        <f>IFERROR(D8/C8-1,"")</f>
-        <v/>
+      <c r="D8" s="11" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
@@ -1441,13 +1410,11 @@
       <c r="C9" s="11" t="n">
         <v>1458115248.22</v>
       </c>
-      <c r="D9" s="11">
-        <f>C9+'Projected P&amp;L FY27'!D19</f>
-        <v/>
-      </c>
-      <c r="E9" s="12">
-        <f>IFERROR(D9/C9-1,"")</f>
-        <v/>
+      <c r="D9" s="11" t="n">
+        <v>1573554048.839</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>0.07916987409597609</v>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
@@ -1465,13 +1432,11 @@
       <c r="C10" s="11" t="n">
         <v>15721313.81</v>
       </c>
-      <c r="D10" s="11">
-        <f>C10</f>
-        <v/>
-      </c>
-      <c r="E10" s="12">
-        <f>IFERROR(D10/C10-1,"")</f>
-        <v/>
+      <c r="D10" s="11" t="n">
+        <v>15721313.81</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
@@ -1486,13 +1451,11 @@
           <t>Sub-total — Shareholders’ funds</t>
         </is>
       </c>
-      <c r="C11" s="16">
-        <f>SUM(C8:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="16">
-        <f>SUM(D8:D10)</f>
-        <v/>
+      <c r="C11" s="16" t="n">
+        <v>1474036562.03</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>1589475362.649</v>
       </c>
       <c r="E11" s="14" t="n"/>
       <c r="F11" s="18" t="inlineStr"/>
@@ -1527,13 +1490,11 @@
       <c r="C13" s="11" t="n">
         <v>89963690.64</v>
       </c>
-      <c r="D13" s="11">
-        <f>C13</f>
-        <v/>
-      </c>
-      <c r="E13" s="12">
-        <f>IFERROR(D13/C13-1,"")</f>
-        <v/>
+      <c r="D13" s="11" t="n">
+        <v>89963690.64</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
@@ -1555,13 +1516,11 @@
       <c r="C14" s="11" t="n">
         <v>94505792</v>
       </c>
-      <c r="D14" s="11">
-        <f>C14*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E14" s="12">
-        <f>IFERROR(D14/C14-1,"")</f>
-        <v/>
+      <c r="D14" s="11" t="n">
+        <v>103956371.2</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -1576,13 +1535,11 @@
           <t>Sub-total — Non-current liabilities</t>
         </is>
       </c>
-      <c r="C15" s="16">
-        <f>SUM(C13:C14)</f>
-        <v/>
-      </c>
-      <c r="D15" s="16">
-        <f>SUM(D13:D14)</f>
-        <v/>
+      <c r="C15" s="16" t="n">
+        <v>184469482.64</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>193920061.84</v>
       </c>
       <c r="E15" s="14" t="n"/>
       <c r="F15" s="18" t="inlineStr"/>
@@ -1617,13 +1574,11 @@
       <c r="C17" s="11" t="n">
         <v>348135361.67</v>
       </c>
-      <c r="D17" s="11">
-        <f>C17</f>
-        <v/>
-      </c>
-      <c r="E17" s="12">
-        <f>IFERROR(D17/C17-1,"")</f>
-        <v/>
+      <c r="D17" s="11" t="n">
+        <v>348135361.67</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
@@ -1661,13 +1616,11 @@
       <c r="C19" s="11" t="n">
         <v>72303716.06999999</v>
       </c>
-      <c r="D19" s="11">
-        <f>C19*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E19" s="12">
-        <f>IFERROR(D19/C19-1,"")</f>
-        <v/>
+      <c r="D19" s="11" t="n">
+        <v>79534087.677</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
@@ -1689,13 +1642,11 @@
       <c r="C20" s="11" t="n">
         <v>495509114.47</v>
       </c>
-      <c r="D20" s="11">
-        <f>C20*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E20" s="12">
-        <f>IFERROR(D20/C20-1,"")</f>
-        <v/>
+      <c r="D20" s="11" t="n">
+        <v>545060025.9170001</v>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
@@ -1717,13 +1668,11 @@
       <c r="C21" s="11" t="n">
         <v>20273486.75</v>
       </c>
-      <c r="D21" s="11">
-        <f>C21*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E21" s="12">
-        <f>IFERROR(D21/C21-1,"")</f>
-        <v/>
+      <c r="D21" s="11" t="n">
+        <v>22300835.425</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
@@ -1738,13 +1687,11 @@
           <t>Sub-total — Current liabilities</t>
         </is>
       </c>
-      <c r="C22" s="16">
-        <f>SUM(C17:C21)</f>
-        <v/>
-      </c>
-      <c r="D22" s="16">
-        <f>SUM(D17:D21)</f>
-        <v/>
+      <c r="C22" s="16" t="n">
+        <v>936221678.96</v>
+      </c>
+      <c r="D22" s="16" t="n">
+        <v>995030310.689</v>
       </c>
       <c r="E22" s="14" t="n"/>
       <c r="F22" s="18" t="inlineStr"/>
@@ -1756,13 +1703,11 @@
           <t>TOTAL — EQUITY AND LIABILITIES</t>
         </is>
       </c>
-      <c r="C23" s="26">
-        <f>C11+C15+C22</f>
-        <v/>
-      </c>
-      <c r="D23" s="26">
-        <f>D11+D15+D22</f>
-        <v/>
+      <c r="C23" s="26" t="n">
+        <v>2594727723.63</v>
+      </c>
+      <c r="D23" s="26" t="n">
+        <v>2778425735.178</v>
       </c>
       <c r="E23" s="24" t="n"/>
       <c r="F23" s="27" t="inlineStr"/>
@@ -1813,13 +1758,11 @@
       <c r="C27" s="11" t="n">
         <v>186880905.31</v>
       </c>
-      <c r="D27" s="11">
-        <f>C27</f>
-        <v/>
-      </c>
-      <c r="E27" s="12">
-        <f>IFERROR(D27/C27-1,"")</f>
-        <v/>
+      <c r="D27" s="11" t="n">
+        <v>186880905.31</v>
+      </c>
+      <c r="E27" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="F27" s="13" t="inlineStr">
         <is>
@@ -1841,13 +1784,11 @@
       <c r="C28" s="11" t="n">
         <v>157195317</v>
       </c>
-      <c r="D28" s="11">
-        <f>C28</f>
-        <v/>
-      </c>
-      <c r="E28" s="12">
-        <f>IFERROR(D28/C28-1,"")</f>
-        <v/>
+      <c r="D28" s="11" t="n">
+        <v>157195317</v>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -1869,13 +1810,11 @@
       <c r="C29" s="11" t="n">
         <v>29044756</v>
       </c>
-      <c r="D29" s="11">
-        <f>C29</f>
-        <v/>
-      </c>
-      <c r="E29" s="12">
-        <f>IFERROR(D29/C29-1,"")</f>
-        <v/>
+      <c r="D29" s="11" t="n">
+        <v>29044756</v>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -1897,13 +1836,11 @@
       <c r="C30" s="11" t="n">
         <v>86514244.73999999</v>
       </c>
-      <c r="D30" s="11">
-        <f>C30</f>
-        <v/>
-      </c>
-      <c r="E30" s="12">
-        <f>IFERROR(D30/C30-1,"")</f>
-        <v/>
+      <c r="D30" s="11" t="n">
+        <v>86514244.73999999</v>
+      </c>
+      <c r="E30" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -1918,13 +1855,11 @@
           <t>Sub-total — Non-current assets</t>
         </is>
       </c>
-      <c r="C31" s="16">
-        <f>SUM(C27:C30)</f>
-        <v/>
-      </c>
-      <c r="D31" s="16">
-        <f>SUM(D27:D30)</f>
-        <v/>
+      <c r="C31" s="16" t="n">
+        <v>459635223.05</v>
+      </c>
+      <c r="D31" s="16" t="n">
+        <v>459635223.05</v>
       </c>
       <c r="E31" s="14" t="n"/>
       <c r="F31" s="18" t="inlineStr"/>
@@ -1959,13 +1894,11 @@
       <c r="C33" s="11" t="n">
         <v>4636862</v>
       </c>
-      <c r="D33" s="11">
-        <f>C33*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E33" s="12">
-        <f>IFERROR(D33/C33-1,"")</f>
-        <v/>
+      <c r="D33" s="11" t="n">
+        <v>5100548.2</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F33" s="13" t="inlineStr">
         <is>
@@ -1987,13 +1920,11 @@
       <c r="C34" s="11" t="n">
         <v>1665625897.28</v>
       </c>
-      <c r="D34" s="11">
-        <f>C34*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E34" s="12">
-        <f>IFERROR(D34/C34-1,"")</f>
-        <v/>
+      <c r="D34" s="11" t="n">
+        <v>1832188487.008</v>
+      </c>
+      <c r="E34" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F34" s="13" t="inlineStr">
         <is>
@@ -2015,13 +1946,11 @@
       <c r="C35" s="11" t="n">
         <v>393603021</v>
       </c>
-      <c r="D35" s="11">
-        <f>C35*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E35" s="12">
-        <f>IFERROR(D35/C35-1,"")</f>
-        <v/>
+      <c r="D35" s="11" t="n">
+        <v>432963323.1</v>
+      </c>
+      <c r="E35" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2043,13 +1972,11 @@
       <c r="C36" s="11" t="n">
         <v>23144280.66</v>
       </c>
-      <c r="D36" s="11">
-        <f>C36*(1+Assumptions!$C$6)</f>
-        <v/>
-      </c>
-      <c r="E36" s="12">
-        <f>IFERROR(D36/C36-1,"")</f>
-        <v/>
+      <c r="D36" s="11" t="n">
+        <v>25458708.726</v>
+      </c>
+      <c r="E36" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
@@ -2071,13 +1998,11 @@
       <c r="C37" s="11" t="n">
         <v>48082440</v>
       </c>
-      <c r="D37" s="11">
-        <f>D23-SUM(D27:D30)-SUM(D33:D36)</f>
-        <v/>
-      </c>
-      <c r="E37" s="12">
-        <f>D37/C37-1</f>
-        <v/>
+      <c r="D37" s="11" t="n">
+        <v>23079445.09400034</v>
+      </c>
+      <c r="E37" s="12" t="n">
+        <v>-0.5200026227038324</v>
       </c>
       <c r="F37" s="13" t="inlineStr">
         <is>
@@ -2092,13 +2017,11 @@
           <t>Sub-total — Current assets</t>
         </is>
       </c>
-      <c r="C38" s="16">
-        <f>SUM(C33:C37)</f>
-        <v/>
-      </c>
-      <c r="D38" s="16">
-        <f>SUM(D33:D37)</f>
-        <v/>
+      <c r="C38" s="16" t="n">
+        <v>2135092500.94</v>
+      </c>
+      <c r="D38" s="16" t="n">
+        <v>2318790512.128</v>
       </c>
       <c r="E38" s="14" t="n"/>
       <c r="F38" s="18" t="inlineStr"/>
@@ -2110,13 +2033,11 @@
           <t>TOTAL — ASSETS</t>
         </is>
       </c>
-      <c r="C39" s="26">
-        <f>C31+C38</f>
-        <v/>
-      </c>
-      <c r="D39" s="26">
-        <f>D31+D38</f>
-        <v/>
+      <c r="C39" s="26" t="n">
+        <v>2594727723.99</v>
+      </c>
+      <c r="D39" s="26" t="n">
+        <v>2778425735.178</v>
       </c>
       <c r="E39" s="24" t="n"/>
       <c r="F39" s="27" t="inlineStr"/>
@@ -2127,9 +2048,8 @@
           <t>Check: Total assets less total equity &amp; liabilities</t>
         </is>
       </c>
-      <c r="D41" s="28">
-        <f>D39-D23</f>
-        <v/>
+      <c r="D41" s="28" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2206,17 +2126,14 @@
           <t>Revenue from operations</t>
         </is>
       </c>
-      <c r="B6" s="30">
-        <f>'Projected P&amp;L FY27'!C6</f>
-        <v/>
-      </c>
-      <c r="C6" s="30">
-        <f>'Projected P&amp;L FY27'!D6</f>
-        <v/>
-      </c>
-      <c r="D6" s="12">
-        <f>IFERROR(C6/B6-1,"")</f>
-        <v/>
+      <c r="B6" s="30" t="n">
+        <v>4898238075.54</v>
+      </c>
+      <c r="C6" s="30" t="n">
+        <v>5388061883.094001</v>
+      </c>
+      <c r="D6" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -2225,17 +2142,14 @@
           <t>Total expenses</t>
         </is>
       </c>
-      <c r="B7" s="30">
-        <f>'Projected P&amp;L FY27'!C16</f>
-        <v/>
-      </c>
-      <c r="C7" s="30">
-        <f>'Projected P&amp;L FY27'!D16</f>
-        <v/>
-      </c>
-      <c r="D7" s="12">
-        <f>IFERROR(C7/B7-1,"")</f>
-        <v/>
+      <c r="B7" s="30" t="n">
+        <v>4767109448.75</v>
+      </c>
+      <c r="C7" s="30" t="n">
+        <v>5243791546.125</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>0.09999394863904221</v>
       </c>
     </row>
     <row r="8">
@@ -2244,17 +2158,14 @@
           <t>Profit before tax</t>
         </is>
       </c>
-      <c r="B8" s="30">
-        <f>'Projected P&amp;L FY27'!C17</f>
-        <v/>
-      </c>
-      <c r="C8" s="30">
-        <f>'Projected P&amp;L FY27'!D17</f>
-        <v/>
-      </c>
-      <c r="D8" s="12">
-        <f>IFERROR(C8/B8-1,"")</f>
-        <v/>
+      <c r="B8" s="30" t="n">
+        <v>141122242.4399996</v>
+      </c>
+      <c r="C8" s="30" t="n">
+        <v>154263952.6190004</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>0.09312288376219824</v>
       </c>
     </row>
     <row r="9">
@@ -2263,17 +2174,14 @@
           <t>Profit after tax</t>
         </is>
       </c>
-      <c r="B9" s="30">
-        <f>'Projected P&amp;L FY27'!C19</f>
-        <v/>
-      </c>
-      <c r="C9" s="30">
-        <f>'Projected P&amp;L FY27'!D19</f>
-        <v/>
-      </c>
-      <c r="D9" s="12">
-        <f>IFERROR(C9/B9-1,"")</f>
-        <v/>
+      <c r="B9" s="30" t="n">
+        <v>170784345.44</v>
+      </c>
+      <c r="C9" s="30" t="n">
+        <v>115438800.6190004</v>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>-0.3240668497947523</v>
       </c>
     </row>
     <row r="10">
@@ -2282,17 +2190,14 @@
           <t>Net worth (incl. interunit)</t>
         </is>
       </c>
-      <c r="B10" s="30">
-        <f>'Projected BS FY27'!C11</f>
-        <v/>
-      </c>
-      <c r="C10" s="30">
-        <f>'Projected BS FY27'!D11</f>
-        <v/>
-      </c>
-      <c r="D10" s="12">
-        <f>IFERROR(C10/B10-1,"")</f>
-        <v/>
+      <c r="B10" s="30" t="n">
+        <v>1474036562.03</v>
+      </c>
+      <c r="C10" s="30" t="n">
+        <v>1589475362.649</v>
+      </c>
+      <c r="D10" s="12" t="n">
+        <v>0.07831474713220232</v>
       </c>
     </row>
     <row r="11">
@@ -2301,17 +2206,14 @@
           <t>Total borrowings (LT+ST)</t>
         </is>
       </c>
-      <c r="B11" s="30">
-        <f>'Projected BS FY27'!C13+'Projected BS FY27'!C17</f>
-        <v/>
-      </c>
-      <c r="C11" s="30">
-        <f>'Projected BS FY27'!D13+'Projected BS FY27'!D17</f>
-        <v/>
-      </c>
-      <c r="D11" s="12">
-        <f>IFERROR(C11/B11-1,"")</f>
-        <v/>
+      <c r="B11" s="30" t="n">
+        <v>438099052.31</v>
+      </c>
+      <c r="C11" s="30" t="n">
+        <v>438099052.31</v>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -2320,17 +2222,14 @@
           <t>Trade receivables</t>
         </is>
       </c>
-      <c r="B12" s="30">
-        <f>'Projected BS FY27'!C34</f>
-        <v/>
-      </c>
-      <c r="C12" s="30">
-        <f>'Projected BS FY27'!D34</f>
-        <v/>
-      </c>
-      <c r="D12" s="12">
-        <f>IFERROR(C12/B12-1,"")</f>
-        <v/>
+      <c r="B12" s="30" t="n">
+        <v>1665625897.28</v>
+      </c>
+      <c r="C12" s="30" t="n">
+        <v>1832188487.008</v>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>0.1000000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -2339,17 +2238,14 @@
           <t>Cash &amp; cash equivalents</t>
         </is>
       </c>
-      <c r="B13" s="30">
-        <f>'Projected BS FY27'!C37</f>
-        <v/>
-      </c>
-      <c r="C13" s="30">
-        <f>'Projected BS FY27'!D37</f>
-        <v/>
-      </c>
-      <c r="D13" s="12">
-        <f>IFERROR(C13/B13-1,"")</f>
-        <v/>
+      <c r="B13" s="30" t="n">
+        <v>48082440</v>
+      </c>
+      <c r="C13" s="30" t="n">
+        <v>23079445.09400034</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>-0.5200026227038324</v>
       </c>
     </row>
     <row r="14">
@@ -2358,17 +2254,14 @@
           <t>Balance sheet total</t>
         </is>
       </c>
-      <c r="B14" s="30">
-        <f>'Projected BS FY27'!C39</f>
-        <v/>
-      </c>
-      <c r="C14" s="30">
-        <f>'Projected BS FY27'!D39</f>
-        <v/>
-      </c>
-      <c r="D14" s="12">
-        <f>IFERROR(C14/B14-1,"")</f>
-        <v/>
+      <c r="B14" s="30" t="n">
+        <v>2594727723.99</v>
+      </c>
+      <c r="C14" s="30" t="n">
+        <v>2778425735.178</v>
+      </c>
+      <c r="D14" s="12" t="n">
+        <v>0.07079664254926965</v>
       </c>
     </row>
     <row r="15">
@@ -2377,17 +2270,14 @@
           <t>Working capital (CA − CL)</t>
         </is>
       </c>
-      <c r="B15" s="30">
-        <f>'Projected BS FY27'!C38-'Projected BS FY27'!C22</f>
-        <v/>
-      </c>
-      <c r="C15" s="30">
-        <f>'Projected BS FY27'!D38-'Projected BS FY27'!D22</f>
-        <v/>
-      </c>
-      <c r="D15" s="12">
-        <f>IFERROR(C15/B15-1,"")</f>
-        <v/>
+      <c r="B15" s="30" t="n">
+        <v>1198870821.98</v>
+      </c>
+      <c r="C15" s="30" t="n">
+        <v>1323760201.439</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>0.1041725073037798</v>
       </c>
     </row>
     <row r="17">
@@ -2403,17 +2293,14 @@
           <t>PBT margin %</t>
         </is>
       </c>
-      <c r="B18" s="32">
-        <f>'Projected P&amp;L FY27'!C17/'Projected P&amp;L FY27'!C6*100</f>
-        <v/>
-      </c>
-      <c r="C18" s="32">
-        <f>'Projected P&amp;L FY27'!D17/'Projected P&amp;L FY27'!D6*100</f>
-        <v/>
-      </c>
-      <c r="D18" s="32">
-        <f>C18-B18</f>
-        <v/>
+      <c r="B18" s="32" t="n">
+        <v>2.881081733138129</v>
+      </c>
+      <c r="C18" s="32" t="n">
+        <v>2.863069429529585</v>
+      </c>
+      <c r="D18" s="32" t="n">
+        <v>-0.01801230360854422</v>
       </c>
     </row>
     <row r="19">
@@ -2422,17 +2309,14 @@
           <t>PAT margin %</t>
         </is>
       </c>
-      <c r="B19" s="32">
-        <f>'Projected P&amp;L FY27'!C19/'Projected P&amp;L FY27'!C6*100</f>
-        <v/>
-      </c>
-      <c r="C19" s="32">
-        <f>'Projected P&amp;L FY27'!D19/'Projected P&amp;L FY27'!D6*100</f>
-        <v/>
-      </c>
-      <c r="D19" s="32">
-        <f>C19-B19</f>
-        <v/>
+      <c r="B19" s="32" t="n">
+        <v>3.486648521492539</v>
+      </c>
+      <c r="C19" s="32" t="n">
+        <v>2.142492107991746</v>
+      </c>
+      <c r="D19" s="32" t="n">
+        <v>-1.344156413500793</v>
       </c>
     </row>
     <row r="20">
@@ -2441,17 +2325,14 @@
           <t>Current ratio (x)</t>
         </is>
       </c>
-      <c r="B20" s="32">
-        <f>'Projected BS FY27'!C38/'Projected BS FY27'!C22</f>
-        <v/>
-      </c>
-      <c r="C20" s="32">
-        <f>'Projected BS FY27'!D38/'Projected BS FY27'!D22</f>
-        <v/>
-      </c>
-      <c r="D20" s="32">
-        <f>C20-B20</f>
-        <v/>
+      <c r="B20" s="32" t="n">
+        <v>2.280541616288744</v>
+      </c>
+      <c r="C20" s="32" t="n">
+        <v>2.330371735633233</v>
+      </c>
+      <c r="D20" s="32" t="n">
+        <v>0.04983011934448944</v>
       </c>
     </row>
     <row r="21">
@@ -2460,17 +2341,14 @@
           <t>Debt / equity (x)</t>
         </is>
       </c>
-      <c r="B21" s="32">
-        <f>('Projected BS FY27'!C13+'Projected BS FY27'!C17)/'Projected BS FY27'!C11</f>
-        <v/>
-      </c>
-      <c r="C21" s="32">
-        <f>('Projected BS FY27'!D13+'Projected BS FY27'!D17)/'Projected BS FY27'!D11</f>
-        <v/>
-      </c>
-      <c r="D21" s="32">
-        <f>C21-B21</f>
-        <v/>
+      <c r="B21" s="32" t="n">
+        <v>0.2972104380549848</v>
+      </c>
+      <c r="C21" s="32" t="n">
+        <v>0.2756249405337554</v>
+      </c>
+      <c r="D21" s="32" t="n">
+        <v>-0.0215854975212294</v>
       </c>
     </row>
     <row r="22">
@@ -2479,17 +2357,14 @@
           <t>Debtor days (on closing TR)</t>
         </is>
       </c>
-      <c r="B22" s="32">
-        <f>'Projected BS FY27'!C34/'Projected P&amp;L FY27'!C6*365</f>
-        <v/>
-      </c>
-      <c r="C22" s="32">
-        <f>'Projected BS FY27'!D34/'Projected P&amp;L FY27'!D6*365</f>
-        <v/>
-      </c>
-      <c r="D22" s="32">
-        <f>C22-B22</f>
-        <v/>
+      <c r="B22" s="32" t="n">
+        <v>124.1167626259524</v>
+      </c>
+      <c r="C22" s="32" t="n">
+        <v>124.1167626259524</v>
+      </c>
+      <c r="D22" s="32" t="n">
+        <v>-2.842170943040401e-14</v>
       </c>
     </row>
     <row r="23">
@@ -2498,17 +2373,14 @@
           <t>Return on net worth %</t>
         </is>
       </c>
-      <c r="B23" s="32">
-        <f>'Projected P&amp;L FY27'!C19/'Projected BS FY27'!C11*100</f>
-        <v/>
-      </c>
-      <c r="C23" s="32">
-        <f>'Projected P&amp;L FY27'!D19/'Projected BS FY27'!D11*100</f>
-        <v/>
-      </c>
-      <c r="D23" s="32">
-        <f>C23-B23</f>
-        <v/>
+      <c r="B23" s="32" t="n">
+        <v>11.58616752387748</v>
+      </c>
+      <c r="C23" s="32" t="n">
+        <v>7.262698330008181</v>
+      </c>
+      <c r="D23" s="32" t="n">
+        <v>-4.3234691938693</v>
       </c>
     </row>
     <row r="25" ht="14" customHeight="1">

</xml_diff>